<commit_message>
Updated Power Budget to rev2
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/EGR314-Power_Budget.xlsx
+++ b/docs/05-Power-Budget/EGR314-Power_Budget.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a531e40cc6beaed5/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="8_{78606173-F688-492F-A36F-4C67BB02F028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFB231FF-BFE9-4A7A-AA1F-62F631A9DFFB}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="8_{78606173-F688-492F-A36F-4C67BB02F028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7288CF1-DA8D-4473-8042-49F6CF8D4ECF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
   <si>
     <t>Team Number:</t>
   </si>
@@ -102,13 +102,7 @@
     <t>Unit</t>
   </si>
   <si>
-    <t>(full part number)</t>
-  </si>
-  <si>
     <t>mA</t>
-  </si>
-  <si>
-    <t>(range)</t>
   </si>
   <si>
     <t>B. Assign each major component above to ONE power rail below. Try to minimize the number of different power rails in the design. 
@@ -127,9 +121,6 @@
     <t>c2. Regulator or Source Choice</t>
   </si>
   <si>
-    <t xml:space="preserve"> -5V Regulator</t>
-  </si>
-  <si>
     <t xml:space="preserve"> +3.3V Power Rail</t>
   </si>
   <si>
@@ -166,48 +157,6 @@
     <t>Total Remaining Current Available on External Power Source 1</t>
   </si>
   <si>
-    <t>External Power Source 2</t>
-  </si>
-  <si>
-    <t>Power Source 2 Selection</t>
-  </si>
-  <si>
-    <t>Battery</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> +9V</t>
-  </si>
-  <si>
-    <t>-9V</t>
-  </si>
-  <si>
-    <t>Power Rails Connected to External Power Source 2</t>
-  </si>
-  <si>
-    <t>Total Remaining Current Available on External Power Source 2</t>
-  </si>
-  <si>
-    <t>E. Calculate Battery Life (if applicable).  For each battery, also check the worst-case lifetime of the battery by indicating the capacity in mAh.</t>
-  </si>
-  <si>
-    <t>Capacity
-(mAh)</t>
-  </si>
-  <si>
-    <t>Required
-By
-Regulators</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> +12V</t>
-  </si>
-  <si>
-    <t>Battery Life</t>
-  </si>
-  <si>
-    <t>hours</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -277,20 +226,23 @@
     <t xml:space="preserve"> -0.3V to 4V</t>
   </si>
   <si>
-    <t>4V to 40V</t>
-  </si>
-  <si>
     <t>Total Remaining Current Available on +9V Rail</t>
   </si>
   <si>
     <t>Total Current Required on +9V Rail</t>
+  </si>
+  <si>
+    <t>LM2575D2T-3.3R4G</t>
+  </si>
+  <si>
+    <t>4.75V to 40V</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -339,10 +291,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
@@ -373,7 +321,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -544,36 +492,7 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -581,7 +500,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -621,9 +540,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -674,77 +590,60 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1098,7 +997,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr defaultColWidth="13.3984375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
@@ -1112,84 +1011,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="55" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
+      <c r="A1" s="60" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="62" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
+      <c r="B2" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="64" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
+      <c r="B3" s="63" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="64" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
+      <c r="B4" s="63" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="64">
-        <v>1</v>
-      </c>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
+      <c r="B5" s="63">
+        <v>2</v>
+      </c>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="57" t="s">
+      <c r="A6" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="59"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="46"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
@@ -1201,7 +1100,7 @@
       <c r="C7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="51" t="s">
+      <c r="D7" s="42" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="8" t="s">
@@ -1220,13 +1119,13 @@
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11"/>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="E8" s="13">
         <v>1</v>
@@ -1239,19 +1138,19 @@
         <v>335</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11"/>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E9" s="13">
         <v>1</v>
@@ -1264,7 +1163,7 @@
         <v>40</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1278,20 +1177,20 @@
       <c r="H10" s="19"/>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="57" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="58"/>
-      <c r="C11" s="58"/>
-      <c r="D11" s="58"/>
-      <c r="E11" s="58"/>
-      <c r="F11" s="58"/>
-      <c r="G11" s="58"/>
-      <c r="H11" s="59"/>
+      <c r="A11" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="46"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="20" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>6</v>
@@ -1299,7 +1198,7 @@
       <c r="C12" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="52" t="s">
+      <c r="D12" s="43" t="s">
         <v>8</v>
       </c>
       <c r="E12" s="8" t="s">
@@ -1308,23 +1207,23 @@
       <c r="F12" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="29" t="s">
+      <c r="G12" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="29" t="s">
+      <c r="H12" s="28" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11"/>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="E13" s="13">
         <v>1</v>
@@ -1337,19 +1236,19 @@
         <v>335</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11"/>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E14" s="13">
         <v>1</v>
@@ -1362,7 +1261,7 @@
         <v>40</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1374,54 +1273,54 @@
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11"/>
-      <c r="B16" s="60" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="56"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
+      <c r="B16" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="51"/>
+      <c r="D16" s="51"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="51"/>
       <c r="G16" s="14">
         <f>SUM(G12:G15)</f>
         <v>375</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11"/>
-      <c r="B17" s="60" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="22">
+      <c r="B17" s="57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="51"/>
+      <c r="D17" s="51"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="21">
         <v>0.25</v>
       </c>
-      <c r="H17" s="22"/>
+      <c r="H17" s="21"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11"/>
-      <c r="B18" s="61" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="56"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
+      <c r="B18" s="58" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="51"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="51"/>
       <c r="G18" s="14">
         <f>G16*(1+G17)</f>
         <v>468.75</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="24"/>
+      <c r="A19" s="23"/>
       <c r="B19" s="16"/>
       <c r="D19" s="12"/>
       <c r="E19" s="13"/>
@@ -1429,17 +1328,17 @@
       <c r="H19" s="19"/>
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="24" t="s">
-        <v>19</v>
+      <c r="A20" s="23" t="s">
+        <v>17</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E20" s="13">
         <v>1</v>
@@ -1452,39 +1351,39 @@
         <v>1000</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11"/>
-      <c r="B21" s="66" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="27">
+      <c r="B21" s="55" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="51"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="26">
         <f>G20-G18</f>
         <v>531.25</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="30"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="33"/>
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="32"/>
     </row>
     <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="20" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>6</v>
@@ -1492,7 +1391,7 @@
       <c r="C23" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="52" t="s">
+      <c r="D23" s="43" t="s">
         <v>8</v>
       </c>
       <c r="E23" s="8" t="s">
@@ -1501,23 +1400,23 @@
       <c r="F23" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G23" s="29" t="s">
+      <c r="G23" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="H23" s="29" t="s">
+      <c r="H23" s="28" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11"/>
       <c r="B24" s="16" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E24" s="13">
         <v>1</v>
@@ -1530,7 +1429,7 @@
         <v>1000</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1542,153 +1441,153 @@
     </row>
     <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11"/>
-      <c r="B26" s="60" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="56"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="56"/>
-      <c r="F26" s="56"/>
+      <c r="B26" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
       <c r="G26" s="14">
         <f>SUM(G24:G25)</f>
         <v>1000</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11"/>
-      <c r="B27" s="60" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="56"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="56"/>
-      <c r="F27" s="56"/>
-      <c r="G27" s="22">
+      <c r="B27" s="57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="21">
         <v>0.25</v>
       </c>
-      <c r="H27" s="22"/>
+      <c r="H27" s="21"/>
     </row>
     <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="23"/>
-      <c r="B28" s="61" t="s">
-        <v>72</v>
-      </c>
-      <c r="C28" s="56"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="56"/>
-      <c r="F28" s="56"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="51"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="51"/>
       <c r="G28" s="14">
         <f>G26*(1+G27)</f>
         <v>1250</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="24"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
+      <c r="A29" s="23"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
       <c r="D29" s="12"/>
       <c r="E29" s="12"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="27"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="26"/>
       <c r="H29" s="14"/>
     </row>
     <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="25" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="25" t="s">
-        <v>56</v>
+      <c r="A30" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>40</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="E30" s="12">
         <v>1</v>
       </c>
-      <c r="F30" s="26">
+      <c r="F30" s="25">
         <v>5000</v>
       </c>
-      <c r="G30" s="27">
+      <c r="G30" s="26">
         <f>E30*F30</f>
         <v>5000</v>
       </c>
       <c r="H30" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="28"/>
-      <c r="B31" s="67" t="s">
-        <v>71</v>
-      </c>
-      <c r="C31" s="68"/>
-      <c r="D31" s="68"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="68"/>
-      <c r="G31" s="27">
+      <c r="A31" s="27"/>
+      <c r="B31" s="59" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" s="48"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="48"/>
+      <c r="G31" s="26">
         <f>G30-G28</f>
         <v>3750</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="30"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="33"/>
+      <c r="A32" s="29"/>
+      <c r="B32" s="30"/>
+      <c r="C32" s="30"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="31"/>
+      <c r="H32" s="32"/>
     </row>
     <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="57" t="s">
-        <v>25</v>
-      </c>
-      <c r="B33" s="58"/>
-      <c r="C33" s="58"/>
-      <c r="D33" s="58"/>
-      <c r="E33" s="58"/>
-      <c r="F33" s="58"/>
-      <c r="G33" s="58"/>
-      <c r="H33" s="59"/>
+      <c r="A33" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33" s="45"/>
+      <c r="C33" s="45"/>
+      <c r="D33" s="45"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="45"/>
+      <c r="G33" s="45"/>
+      <c r="H33" s="46"/>
     </row>
     <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="69"/>
-      <c r="B34" s="68"/>
-      <c r="C34" s="68"/>
-      <c r="D34" s="68"/>
-      <c r="E34" s="68"/>
-      <c r="F34" s="68"/>
-      <c r="G34" s="68"/>
-      <c r="H34" s="70"/>
+      <c r="A34" s="47"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="49"/>
     </row>
     <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="57" t="s">
-        <v>26</v>
-      </c>
-      <c r="B35" s="58"/>
-      <c r="C35" s="58"/>
-      <c r="D35" s="58"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="58"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="59"/>
+      <c r="A35" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" s="45"/>
+      <c r="C35" s="45"/>
+      <c r="D35" s="45"/>
+      <c r="E35" s="45"/>
+      <c r="F35" s="45"/>
+      <c r="G35" s="45"/>
+      <c r="H35" s="46"/>
     </row>
     <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="20" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>6</v>
@@ -1696,96 +1595,96 @@
       <c r="C36" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D36" s="52" t="s">
+      <c r="D36" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="E36" s="34" t="s">
-        <v>28</v>
+      <c r="E36" s="33" t="s">
+        <v>25</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G36" s="29" t="s">
+      <c r="G36" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="H36" s="29" t="s">
+      <c r="H36" s="28" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>30</v>
+      <c r="A37" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37" s="24" t="s">
+        <v>27</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="F37" s="26">
+        <v>44</v>
+      </c>
+      <c r="F37" s="25">
         <v>15000</v>
       </c>
-      <c r="G37" s="36">
+      <c r="G37" s="35">
         <f>F37</f>
         <v>15000</v>
       </c>
-      <c r="H37" s="37" t="s">
-        <v>14</v>
+      <c r="H37" s="36" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="38"/>
-      <c r="B38" s="25"/>
-      <c r="C38" s="25"/>
+      <c r="A38" s="37"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
       <c r="D38" s="12"/>
       <c r="E38" s="12"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="39"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="38"/>
     </row>
     <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="73" t="s">
-        <v>32</v>
-      </c>
-      <c r="B39" s="25" t="s">
-        <v>55</v>
-      </c>
-      <c r="C39" s="25" t="s">
-        <v>56</v>
+      <c r="A39" s="53" t="s">
+        <v>29</v>
+      </c>
+      <c r="B39" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" s="24" t="s">
+        <v>40</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="F39" s="26">
+        <v>43</v>
+      </c>
+      <c r="F39" s="25">
         <v>5000</v>
       </c>
-      <c r="G39" s="27">
+      <c r="G39" s="26">
         <f>F39</f>
         <v>5000</v>
       </c>
       <c r="H39" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="74"/>
+      <c r="A40" s="54"/>
       <c r="B40" s="16" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C40" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="E40" s="13">
         <v>1</v>
@@ -1793,318 +1692,101 @@
       <c r="F40">
         <v>1000</v>
       </c>
-      <c r="G40" s="27">
+      <c r="G40" s="26">
         <f t="shared" ref="G40" si="3">E40*F40</f>
         <v>1000</v>
       </c>
       <c r="H40" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="38"/>
-      <c r="B41" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="C41" s="56"/>
-      <c r="D41" s="56"/>
-      <c r="E41" s="56"/>
-      <c r="F41" s="56"/>
-      <c r="G41" s="36">
+      <c r="A41" s="37"/>
+      <c r="B41" s="55" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" s="51"/>
+      <c r="D41" s="51"/>
+      <c r="E41" s="51"/>
+      <c r="F41" s="51"/>
+      <c r="G41" s="35">
         <f>G37-SUM(G39:G40)</f>
         <v>9000</v>
       </c>
-      <c r="H41" s="37" t="s">
-        <v>14</v>
+      <c r="H41" s="36" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="38"/>
+      <c r="A42" s="37"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="18"/>
       <c r="E42" s="18"/>
       <c r="F42" s="18"/>
-      <c r="G42" s="40"/>
-      <c r="H42" s="41"/>
+      <c r="G42" s="39"/>
+      <c r="H42" s="40"/>
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" s="52" t="s">
-        <v>8</v>
-      </c>
-      <c r="E43" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="G43" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="H43" s="29" t="s">
-        <v>12</v>
-      </c>
+      <c r="A43" s="56" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="51"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="51"/>
+      <c r="E43" s="51"/>
+      <c r="F43" s="51"/>
+      <c r="G43" s="41"/>
+      <c r="H43" s="41"/>
     </row>
     <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B44" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C44" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E44" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F44" s="26">
-        <v>500</v>
-      </c>
-      <c r="G44" s="36">
-        <v>500</v>
-      </c>
-      <c r="H44" s="37" t="s">
-        <v>14</v>
-      </c>
+      <c r="A44" s="50" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="51"/>
+      <c r="C44" s="51"/>
+      <c r="D44" s="51"/>
+      <c r="E44" s="51"/>
+      <c r="F44" s="51"/>
+      <c r="G44" s="51"/>
+      <c r="H44" s="51"/>
     </row>
     <row r="45" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="38"/>
-      <c r="B45" s="25"/>
-      <c r="C45" s="25"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="27"/>
-      <c r="H45" s="39"/>
-    </row>
-    <row r="46" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="73" t="s">
-        <v>39</v>
-      </c>
-      <c r="B46" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="C46" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E46" s="12">
-        <v>1</v>
-      </c>
-      <c r="F46" s="26">
-        <v>500</v>
-      </c>
-      <c r="G46" s="27">
-        <f>E46*F46</f>
-        <v>500</v>
-      </c>
-      <c r="H46" s="15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="74"/>
-      <c r="B47" s="25"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="15"/>
-    </row>
-    <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="74"/>
-      <c r="B48" s="16"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="13"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="15"/>
-    </row>
-    <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="38"/>
-      <c r="B49" s="66" t="s">
-        <v>40</v>
-      </c>
-      <c r="C49" s="56"/>
-      <c r="D49" s="56"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="36">
-        <f>G44-SUM(G46:G48)</f>
-        <v>0</v>
-      </c>
-      <c r="H49" s="37" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="23"/>
-      <c r="B50" s="16"/>
-      <c r="D50" s="42"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="16"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="43"/>
-    </row>
-    <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="57" t="s">
-        <v>41</v>
-      </c>
-      <c r="B51" s="58"/>
-      <c r="C51" s="58"/>
-      <c r="D51" s="58"/>
-      <c r="E51" s="58"/>
-      <c r="F51" s="75"/>
-      <c r="G51" s="44"/>
-      <c r="H51" s="44"/>
-    </row>
-    <row r="52" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="45"/>
-      <c r="B52" s="46" t="s">
-        <v>6</v>
-      </c>
-      <c r="C52" s="46" t="s">
-        <v>7</v>
-      </c>
-      <c r="D52" s="53" t="s">
-        <v>8</v>
-      </c>
-      <c r="E52" s="47"/>
-      <c r="F52" s="48" t="s">
-        <v>42</v>
-      </c>
-      <c r="G52" s="54" t="s">
-        <v>43</v>
-      </c>
-      <c r="H52" s="49"/>
-    </row>
-    <row r="53" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="11"/>
-      <c r="B53" t="s">
-        <v>36</v>
-      </c>
-      <c r="C53" t="s">
-        <v>13</v>
-      </c>
-      <c r="D53" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="E53" s="13"/>
-      <c r="F53" s="16">
-        <v>500</v>
-      </c>
-      <c r="G53" s="14">
-        <f>SUM(G46:G48)</f>
-        <v>500</v>
-      </c>
-      <c r="H53" s="14"/>
-    </row>
-    <row r="54" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="11"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="G54" s="14">
-        <f>F53/G53</f>
-        <v>1</v>
-      </c>
-      <c r="H54" s="15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="76" t="s">
-        <v>47</v>
-      </c>
-      <c r="B55" s="56"/>
-      <c r="C55" s="56"/>
-      <c r="D55" s="56"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="56"/>
-      <c r="G55" s="50"/>
-      <c r="H55" s="50"/>
-    </row>
-    <row r="56" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="B56" s="56"/>
-      <c r="C56" s="56"/>
-      <c r="D56" s="56"/>
-      <c r="E56" s="56"/>
-      <c r="F56" s="56"/>
-      <c r="G56" s="56"/>
-      <c r="H56" s="56"/>
-    </row>
-    <row r="57" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="72" t="s">
-        <v>49</v>
-      </c>
-      <c r="B57" s="56"/>
-      <c r="C57" s="56"/>
-      <c r="D57" s="56"/>
-      <c r="E57" s="56"/>
-      <c r="F57" s="56"/>
-      <c r="G57" s="56"/>
-      <c r="H57" s="56"/>
-    </row>
-    <row r="58" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="A45" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" s="51"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="51"/>
+      <c r="E45" s="51"/>
+      <c r="F45" s="51"/>
+      <c r="G45" s="51"/>
+      <c r="H45" s="51"/>
+    </row>
+    <row r="46" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="67" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="A33:H33"/>
-    <mergeCell ref="A34:H34"/>
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A57:H57"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="A51:F51"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B31:F31"/>
+  <mergeCells count="23">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A11:H11"/>
@@ -2115,6 +1797,19 @@
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <conditionalFormatting sqref="G21 G31">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>